<commit_message>
Site rebuild Thu Feb 21 15:29:39 CET 2019
</commit_message>
<xml_diff>
--- a/LMI/annuaire/people.xlsx
+++ b/LMI/annuaire/people.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/colin/Travail/Site LMI/Site LMI/content/annuaire/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{EBEAA0DB-BA5A-974C-A432-1FE727621755}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D805135A-D86D-C545-BD82-1D69597D9CBC}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="38400" windowHeight="21140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="185">
   <si>
     <t>JOURNET-GAUTIER</t>
   </si>
@@ -563,6 +563,18 @@
   </si>
   <si>
     <t>T-UCBL</t>
+  </si>
+  <si>
+    <t>DOI</t>
+  </si>
+  <si>
+    <t>10.1016/j.jct.2018.11.015</t>
+  </si>
+  <si>
+    <t>10.4028/www.scientific.net/MSF.740-742.177</t>
+  </si>
+  <si>
+    <t>10.1016/j.jcrysgro.2018.11.034,10.1016/j.apsusc.2017.08.220,10.1063/1.3518275,10.1016/j.jcrysgro.2017.03.018,10.1002/pssa.201600428,10.1038/srep43069</t>
   </si>
 </sst>
 </file>
@@ -1415,7 +1427,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
@@ -1428,7 +1440,7 @@
     <col min="9" max="9" width="26.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>76</v>
       </c>
@@ -1456,8 +1468,11 @@
       <c r="I1" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1477,7 +1492,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -1497,7 +1512,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -1517,7 +1532,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>116</v>
       </c>
@@ -1537,7 +1552,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -1566,7 +1581,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>117</v>
       </c>
@@ -1586,7 +1601,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>41</v>
       </c>
@@ -1606,7 +1621,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>42</v>
       </c>
@@ -1626,7 +1641,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -1645,8 +1660,11 @@
       <c r="F10" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J10" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -1666,7 +1684,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>45</v>
       </c>
@@ -1686,7 +1704,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>46</v>
       </c>
@@ -1706,7 +1724,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>47</v>
       </c>
@@ -1726,7 +1744,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>48</v>
       </c>
@@ -1746,7 +1764,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>118</v>
       </c>
@@ -1766,7 +1784,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>50</v>
       </c>
@@ -1786,7 +1804,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -1806,7 +1824,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>52</v>
       </c>
@@ -1826,7 +1844,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>53</v>
       </c>
@@ -1845,8 +1863,11 @@
       <c r="F20" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="J20" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>54</v>
       </c>
@@ -1866,7 +1887,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>55</v>
       </c>
@@ -1886,7 +1907,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>56</v>
       </c>
@@ -1906,7 +1927,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>57</v>
       </c>
@@ -1926,7 +1947,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -1946,7 +1967,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>59</v>
       </c>
@@ -1966,7 +1987,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>60</v>
       </c>
@@ -1986,7 +2007,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>0</v>
       </c>
@@ -2006,7 +2027,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>61</v>
       </c>
@@ -2026,7 +2047,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>62</v>
       </c>
@@ -2046,7 +2067,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>63</v>
       </c>
@@ -2066,7 +2087,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>64</v>
       </c>
@@ -2086,7 +2107,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -2105,8 +2126,11 @@
       <c r="F33" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="J33" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>66</v>
       </c>
@@ -2126,7 +2150,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>67</v>
       </c>
@@ -2146,7 +2170,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>119</v>
       </c>
@@ -2166,7 +2190,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>68</v>
       </c>
@@ -2186,7 +2210,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>69</v>
       </c>
@@ -2206,7 +2230,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>70</v>
       </c>
@@ -2226,7 +2250,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>71</v>
       </c>
@@ -2246,7 +2270,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>72</v>
       </c>
@@ -2266,7 +2290,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>73</v>
       </c>
@@ -2286,7 +2310,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>74</v>
       </c>
@@ -2309,6 +2333,9 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="I6" r:id="rId1" xr:uid="{17210D97-5C56-C349-8233-DCF311EF75CF}"/>
+    <hyperlink ref="J33" r:id="rId2" tooltip="Persistent link using digital object identifier" display="https://doi.org/10.1016/j.jct.2018.11.015" xr:uid="{1076193C-FDD7-1342-AB36-DF2385B1D3AB}"/>
+    <hyperlink ref="J20" r:id="rId3" tooltip="Persistent link using digital object identifier" display="https://doi.org/10.1016/j.jcrysgro.2018.11.034" xr:uid="{FDCEF42B-9F67-434D-B9EA-096A5634796E}"/>
+    <hyperlink ref="J10" r:id="rId4" display="https://doi.org/10.4028/www.scientific.net/MSF.740-742.177" xr:uid="{FC10D198-F188-5A44-A826-58720D6A5E14}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>